<commit_message>
DESKTOP Phase 2: sidebar shell built to the approved mock (web-only; one TAB_META map, lens order, foot with long-tail/hide/sign-out); pins + logs
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/desktop/docs/MK-desktop-audit-v1-2026-08-03.xlsx
+++ b/desktop/docs/MK-desktop-audit-v1-2026-08-03.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -688,6 +688,40 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="50" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Desktop mock v1 APPROVED (founder: "I like it"). Phase 2 build began.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Phase 2 milestone: the SIDEBAR SHELL is built — web-only branch in the tabs layout renders DesktopSidebar (same TAB_META map, lens order preserved, long-tail + Hide balances + Sign out in the foot); the bottom bar untouched on phones. Web export green; phone suite green. NEXT: Home and Plan two-column layouts to the approved windows.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Build log</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Desktop docs APPROVED (logged); width system: web canvas caps at 1160px centered (approved UX rule)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/desktop/docs/MK-desktop-audit-v1-2026-08-03.xlsx
+++ b/desktop/docs/MK-desktop-audit-v1-2026-08-03.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -722,6 +722,23 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>ALL THREE DESKTOP DOCS APPROVED by the founder ("consider docs approved") — the derived PRD (180 criteria + NFR verdicts + desktop-only requirements), the UX design file (derived rules + 9 desktop-new), and this audit structure. The build proceeds against them as the approved spec.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Desktop: Plan hub two-column interior built to approved shell mock — inline sandbox (one-brain simulate + shared adoptPlan w/ preview), 6 pins, suite 1394 green, web export green
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/desktop/docs/MK-desktop-audit-v1-2026-08-03.xlsx
+++ b/desktop/docs/MK-desktop-audit-v1-2026-08-03.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -739,6 +739,18 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Phase 2 milestone: PLAN TWO-COLUMN INTERIOR BUILT to the approved shell mock — verdict + next-decision + ranked decisions LEFT (1.15) | INLINE sandbox + saved scenarios + revert + sharpen meter RIGHT (0.85). The sandbox is new: dials (retire age / save / spend; retired: spend / plan-to age) re-run the SAME simulate() the verdict uses, patched only on moved dials so at rest sandbox % = hub % exactly; "Use as my plan" previews the exact numbers then writes through the one shared adoptPlan (revert card appears). Phone untouched (12/12 v9 pins green). 6 new desktop pins; suite 1,394 green; tsc clean; web export green. NEXT: Home two-column (glance LEFT | what-needs-you + investments table RIGHT).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Desktop: Home two-column interior built — glance left, chief-of-staff + investments table right (agreement-pinned rows), banners full-width; 3 pins, suite 1397 green, web export green
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/desktop/docs/MK-desktop-audit-v1-2026-08-03.xlsx
+++ b/desktop/docs/MK-desktop-audit-v1-2026-08-03.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -751,6 +751,18 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Phase 2 milestone: HOME TWO-COLUMN INTERIOR BUILT to the approved shell mock — glance LEFT (net-worth line + will-my-money-last gauge + this-month cash flow; retired lens leads with the paycheck card) | chief-of-staff what-needs-you + the NEW investments TABLE RIGHT (class rows from assetAllocation over exactly the accounts investmentsTotal counts — sum pinned equal; validated class colors/labels/liquidity order; rows + See-your-growth open Performance). Connection banners (broken/stale/offline) and milestone stay full-width above the columns. Phone untouched. FIDELITY NOTE vs mock: v1 renders the investments glance card + rows as adjacent cards (mock draws one merged card with hover actions; hover pass + vs-market line inside the table header come with the Performance desktop pane). 3 new pins; suite 1,397 green; tsc clean; web export green. NEXT: Net worth real table · Performance two-pane · Cash flow grid+calendar.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>